<commit_message>
Added csv of normalized replicate averages for each experiment
</commit_message>
<xml_diff>
--- a/Orthobunya_metadata.xlsx
+++ b/Orthobunya_metadata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charligeer/Documents/Lab_Projects/MG_Assays/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charligeer/Documents/Lab_Projects/Repos/Bunya-50-N-experiments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42935240-9802-5A4B-96B4-03F599166963}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9E813C7-CF0E-AA41-88E7-F2B9288B0D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{4C84D9B9-C079-7D4A-BC41-BD4A03A17175}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{4C84D9B9-C079-7D4A-BC41-BD4A03A17175}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="197">
   <si>
     <t>Pct_ID_BUNV_N</t>
   </si>
@@ -624,6 +624,9 @@
   </si>
   <si>
     <t>https://pubmed.ncbi.nlm.nih.gov/23988729/</t>
+  </si>
+  <si>
+    <t>Pct_ID_KAIRI_N</t>
   </si>
 </sst>
 </file>
@@ -1057,23 +1060,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F356077-F51D-5940-97A1-1657D7AA6866}">
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="83" style="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="15" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.1640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20.5" style="1" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="10.83203125" style="1"/>
+    <col min="4" max="5" width="14.6640625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="25.83203125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="15" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.1640625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="20.5" style="1" customWidth="1"/>
+    <col min="12" max="12" width="11.83203125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -1087,31 +1090,34 @@
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>59</v>
       </c>
@@ -1124,32 +1130,35 @@
       <c r="D2" s="3">
         <v>44</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="3">
+        <v>63.2</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K2" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L2" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>60</v>
       </c>
@@ -1162,32 +1171,35 @@
       <c r="D3" s="3">
         <v>46.6</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3">
+        <v>66.5</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="K3" s="8" t="s">
         <v>177</v>
       </c>
-      <c r="K3" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L3" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>61</v>
       </c>
@@ -1200,32 +1212,35 @@
       <c r="D4" s="3">
         <v>47.4</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="3">
+        <v>71.2</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="I4" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="J4" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K4" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L4" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>62</v>
       </c>
@@ -1238,15 +1253,18 @@
       <c r="D5" s="3">
         <v>47.4</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>63</v>
       </c>
@@ -1259,15 +1277,18 @@
       <c r="D6" s="3">
         <v>58.5</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="3">
+        <v>53.2</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>64</v>
       </c>
@@ -1280,15 +1301,18 @@
       <c r="D7" s="3">
         <v>61.1</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="3">
+        <v>52.4</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>65</v>
       </c>
@@ -1301,15 +1325,18 @@
       <c r="D8" s="3">
         <v>64.8</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="3">
+        <v>47.4</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>66</v>
       </c>
@@ -1322,15 +1349,18 @@
       <c r="D9" s="3">
         <v>67.2</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="3">
+        <v>47.6</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>67</v>
       </c>
@@ -1343,32 +1373,35 @@
       <c r="D10" s="3">
         <v>74</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="3">
+        <v>46.6</v>
+      </c>
+      <c r="F10" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="I10" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="K10" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="K10" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L10" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>68</v>
       </c>
@@ -1381,32 +1414,35 @@
       <c r="D11" s="3">
         <v>74.5</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="3">
+        <v>47.9</v>
+      </c>
+      <c r="F11" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="G11" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="H11" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="I11" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="J11" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="K11" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="K11" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L11" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>69</v>
       </c>
@@ -1419,32 +1455,35 @@
       <c r="D12" s="3">
         <v>82.6</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="3">
+        <v>45.7</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="F12" s="4" t="s">
+      <c r="G12" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="J12" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="K12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K12" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L12" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>127</v>
       </c>
@@ -1457,15 +1496,18 @@
       <c r="D13" s="3">
         <v>47.4</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="3">
+        <v>100</v>
+      </c>
+      <c r="F13" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F13" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>163</v>
       </c>
@@ -1478,32 +1520,35 @@
       <c r="D14" s="3">
         <v>36.700000000000003</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="3">
+        <v>37</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="G14" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="H14" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="J14" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K14" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L14" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M14" s="1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>164</v>
       </c>
@@ -1516,32 +1561,35 @@
       <c r="D15" s="3">
         <v>32.5</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="3">
+        <v>27.7</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="G15" s="4" t="s">
+      <c r="H15" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H15" s="1" t="s">
+      <c r="I15" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K15" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L15" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M15" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>165</v>
       </c>
@@ -1554,15 +1602,18 @@
       <c r="D16" s="3">
         <v>43.2</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3">
+        <v>70.8</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="G16" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>166</v>
       </c>
@@ -1575,15 +1626,18 @@
       <c r="D17" s="3">
         <v>21.4</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="3">
+        <v>30.9</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="F17" s="4" t="s">
+      <c r="G17" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>167</v>
       </c>
@@ -1596,15 +1650,18 @@
       <c r="D18" s="3">
         <v>44</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="3">
+        <v>70</v>
+      </c>
+      <c r="F18" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F18" s="4" t="s">
+      <c r="G18" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>169</v>
       </c>
@@ -1617,32 +1674,35 @@
       <c r="D19" s="1">
         <v>100</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="1">
+        <v>47.4</v>
+      </c>
+      <c r="F19" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="F19" s="4" t="s">
+      <c r="G19" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="G19" s="4" t="s">
+      <c r="H19" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="K19" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K19" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L19" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M19" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>170</v>
       </c>
@@ -1655,32 +1715,35 @@
       <c r="D20" s="1">
         <v>41.9</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="1">
+        <v>45.1</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="G20" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="H20" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="I20" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="J20" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="J20" s="1" t="s">
+      <c r="K20" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="L20" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="L20" s="1" t="s">
+      <c r="M20" s="1" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>219</v>
       </c>
@@ -1693,32 +1756,35 @@
       <c r="D21" s="1">
         <v>43.2</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="1">
+        <v>71.7</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="F21" s="4" t="s">
+      <c r="G21" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="G21" s="4" t="s">
+      <c r="H21" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H21" s="1" t="s">
+      <c r="I21" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="J21" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J21" s="1" t="s">
+      <c r="K21" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K21" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L21" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M21" s="1" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>221</v>
       </c>
@@ -1731,32 +1797,35 @@
       <c r="D22" s="1">
         <v>42.3</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="1">
+        <v>69.5</v>
+      </c>
+      <c r="F22" t="s">
         <v>70</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="I22" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="J22" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K22" s="7" t="s">
+      <c r="L22" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="L22" s="1" t="s">
+      <c r="M22" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>222</v>
       </c>
@@ -1769,32 +1838,35 @@
       <c r="D23" s="1">
         <v>42.7</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="1">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="F23" t="s">
         <v>69</v>
       </c>
-      <c r="F23" s="4" t="s">
+      <c r="G23" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="G23" s="4" t="s">
+      <c r="H23" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="I23" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="J23" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K23" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L23" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M23" s="1" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>223</v>
       </c>
@@ -1807,32 +1879,35 @@
       <c r="D24" s="1">
         <v>38.9</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="1">
+        <v>63.9</v>
+      </c>
+      <c r="F24" t="s">
         <v>68</v>
       </c>
-      <c r="F24" s="4" t="s">
+      <c r="G24" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="G24" s="4" t="s">
+      <c r="H24" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H24" s="1" t="s">
+      <c r="I24" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="J24" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K24" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L24" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>224</v>
       </c>
@@ -1845,32 +1920,35 @@
       <c r="D25" s="1">
         <v>44</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="1">
+        <v>71.7</v>
+      </c>
+      <c r="F25" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="4" t="s">
+      <c r="G25" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="G25" s="4" t="s">
+      <c r="H25" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="J25" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J25" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K25" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L25" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M25" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>225</v>
       </c>
@@ -1883,32 +1961,35 @@
       <c r="D26" s="1">
         <v>86</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="1">
+        <v>46.2</v>
+      </c>
+      <c r="F26" t="s">
         <v>89</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="G26" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="H26" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I26" s="5" t="s">
+      <c r="J26" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J26" s="5" t="s">
+      <c r="K26" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K26" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L26" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M26" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>226</v>
       </c>
@@ -1921,32 +2002,35 @@
       <c r="D27" s="1">
         <v>89.8</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="1">
+        <v>47.4</v>
+      </c>
+      <c r="F27" t="s">
         <v>59</v>
       </c>
-      <c r="F27" s="4" t="s">
+      <c r="G27" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G27" s="4" t="s">
+      <c r="H27" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H27" s="1" t="s">
+      <c r="I27" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I27" s="5" t="s">
+      <c r="J27" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J27" s="5" t="s">
+      <c r="K27" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K27" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L27" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M27" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>227</v>
       </c>
@@ -1959,32 +2043,35 @@
       <c r="D28" s="1">
         <v>90.2</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="1">
+        <v>47</v>
+      </c>
+      <c r="F28" t="s">
         <v>60</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="G28" s="4" t="s">
         <v>132</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="H28" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H28" s="1" t="s">
+      <c r="I28" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="J28" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J28" s="5" t="s">
+      <c r="K28" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K28" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L28" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M28" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>228</v>
       </c>
@@ -1997,32 +2084,35 @@
       <c r="D29" s="1">
         <v>89.8</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="1">
+        <v>47</v>
+      </c>
+      <c r="F29" t="s">
         <v>61</v>
       </c>
-      <c r="F29" s="4" t="s">
+      <c r="G29" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="G29" s="4" t="s">
+      <c r="H29" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H29" s="1" t="s">
+      <c r="I29" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I29" s="5" t="s">
+      <c r="J29" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="K29" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K29" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L29" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M29" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>229</v>
       </c>
@@ -2035,32 +2125,35 @@
       <c r="D30" s="1">
         <v>90.2</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="1">
+        <v>46.6</v>
+      </c>
+      <c r="F30" t="s">
         <v>62</v>
       </c>
-      <c r="F30" s="4" t="s">
+      <c r="G30" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="G30" s="4" t="s">
+      <c r="H30" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H30" s="1" t="s">
+      <c r="I30" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I30" s="5" t="s">
+      <c r="J30" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J30" s="5" t="s">
+      <c r="K30" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K30" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L30" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M30" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>230</v>
       </c>
@@ -2073,15 +2166,18 @@
       <c r="D31" s="1">
         <v>45.7</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="1">
+        <v>63.5</v>
+      </c>
+      <c r="F31" t="s">
         <v>71</v>
       </c>
-      <c r="F31" s="4" t="s">
+      <c r="G31" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G31" s="4"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H31" s="4"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>231</v>
       </c>
@@ -2094,17 +2190,20 @@
       <c r="D32" s="1">
         <v>38.9</v>
       </c>
-      <c r="E32" t="s">
+      <c r="E32" s="1">
+        <v>67</v>
+      </c>
+      <c r="F32" t="s">
         <v>63</v>
       </c>
-      <c r="F32" s="4" t="s">
+      <c r="G32" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>232</v>
       </c>
@@ -2117,17 +2216,20 @@
       <c r="D33" s="1">
         <v>44.9</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="1">
+        <v>73</v>
+      </c>
+      <c r="F33" t="s">
         <v>64</v>
       </c>
-      <c r="F33" s="4" t="s">
+      <c r="G33" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="G33" s="4" t="s">
+      <c r="H33" s="4" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>233</v>
       </c>
@@ -2140,32 +2242,35 @@
       <c r="D34" s="1">
         <v>83</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="1">
+        <v>45.7</v>
+      </c>
+      <c r="F34" t="s">
         <v>72</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="G34" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="G34" s="4" t="s">
+      <c r="H34" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="H34" s="1" t="s">
+      <c r="I34" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I34" s="5" t="s">
+      <c r="J34" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J34" s="5" t="s">
+      <c r="K34" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K34" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L34" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M34" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>234</v>
       </c>
@@ -2178,32 +2283,35 @@
       <c r="D35" s="1">
         <v>82.6</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E35" s="1">
+        <v>46.6</v>
+      </c>
+      <c r="F35" t="s">
         <v>73</v>
       </c>
-      <c r="F35" s="4" t="s">
+      <c r="G35" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="G35" s="4" t="s">
+      <c r="H35" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H35" s="1" t="s">
+      <c r="I35" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I35" s="5" t="s">
+      <c r="J35" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J35" s="5" t="s">
+      <c r="K35" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K35" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L35" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M35" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>235</v>
       </c>
@@ -2216,32 +2324,35 @@
       <c r="D36" s="1">
         <v>80.400000000000006</v>
       </c>
-      <c r="E36" t="s">
+      <c r="E36" s="1">
+        <v>47</v>
+      </c>
+      <c r="F36" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="G36" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="G36" s="4" t="s">
+      <c r="H36" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="I36" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I36" s="5" t="s">
+      <c r="J36" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J36" s="5" t="s">
+      <c r="K36" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K36" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L36" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M36" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>236</v>
       </c>
@@ -2254,32 +2365,35 @@
       <c r="D37" s="1">
         <v>98.7</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E37" s="1">
+        <v>47.9</v>
+      </c>
+      <c r="F37" t="s">
         <v>65</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="G37" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="H37" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H37" s="1" t="s">
+      <c r="I37" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I37" s="1" t="s">
+      <c r="J37" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="J37" s="1" t="s">
+      <c r="K37" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="K37" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L37" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M37" s="1" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>237</v>
       </c>
@@ -2292,32 +2406,35 @@
       <c r="D38" s="1">
         <v>85.1</v>
       </c>
-      <c r="E38" t="s">
+      <c r="E38" s="1">
+        <v>46.2</v>
+      </c>
+      <c r="F38" t="s">
         <v>75</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="G38" s="4" t="s">
+      <c r="H38" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="I38" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I38" s="5" t="s">
+      <c r="J38" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J38" s="5" t="s">
+      <c r="K38" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K38" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L38" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M38" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>238</v>
       </c>
@@ -2330,32 +2447,35 @@
       <c r="D39" s="1">
         <v>42.7</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E39" s="1">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="F39" t="s">
         <v>76</v>
       </c>
-      <c r="F39" s="4" t="s">
+      <c r="G39" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="G39" s="4" t="s">
+      <c r="H39" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="I39" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>193</v>
       </c>
       <c r="J39" s="1" t="s">
         <v>193</v>
       </c>
       <c r="K39" s="1" t="s">
-        <v>162</v>
+        <v>193</v>
       </c>
       <c r="L39" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M39" s="1" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="1">
         <v>239</v>
       </c>
@@ -2368,32 +2488,35 @@
       <c r="D40" s="1">
         <v>43.2</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E40" s="1">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="F40" t="s">
         <v>66</v>
       </c>
-      <c r="F40" s="4" t="s">
+      <c r="G40" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G40" s="4" t="s">
+      <c r="H40" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H40" s="1" t="s">
+      <c r="I40" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I40" s="1" t="s">
+      <c r="J40" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J40" s="1" t="s">
+      <c r="K40" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K40" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L40" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M40" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="1">
         <v>240</v>
       </c>
@@ -2406,32 +2529,35 @@
       <c r="D41" s="1">
         <v>83</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E41" s="1">
+        <v>48.3</v>
+      </c>
+      <c r="F41" t="s">
         <v>77</v>
       </c>
-      <c r="F41" s="4" t="s">
+      <c r="G41" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="G41" s="4" t="s">
+      <c r="H41" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="I41" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I41" s="5" t="s">
+      <c r="J41" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J41" s="5" t="s">
+      <c r="K41" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K41" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L41" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M41" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="1">
         <v>241</v>
       </c>
@@ -2444,29 +2570,32 @@
       <c r="D42" s="1">
         <v>32.9</v>
       </c>
-      <c r="E42" t="s">
+      <c r="E42" s="1">
+        <v>54.1</v>
+      </c>
+      <c r="F42" t="s">
         <v>78</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="G42" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="H42" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H42" s="1" t="s">
+      <c r="I42" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I42" s="1" t="s">
+      <c r="J42" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="J42" s="1" t="s">
+      <c r="K42" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K42" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L42" s="1" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="1">
         <v>242</v>
       </c>
@@ -2479,32 +2608,35 @@
       <c r="D43" s="1">
         <v>44</v>
       </c>
-      <c r="E43" t="s">
+      <c r="E43" s="1">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="F43" t="s">
         <v>79</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="G43" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G43" s="4" t="s">
+      <c r="H43" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H43" s="1" t="s">
+      <c r="I43" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I43" s="1" t="s">
+      <c r="J43" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J43" s="1" t="s">
+      <c r="K43" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K43" s="1" t="s">
-        <v>162</v>
-      </c>
       <c r="L43" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M43" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="1">
         <v>243</v>
       </c>
@@ -2517,32 +2649,35 @@
       <c r="D44" s="1">
         <v>86.4</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="1">
+        <v>47.4</v>
+      </c>
+      <c r="F44" t="s">
         <v>80</v>
       </c>
-      <c r="F44" s="4" t="s">
+      <c r="G44" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="G44" s="6" t="s">
+      <c r="H44" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H44" s="5" t="s">
+      <c r="I44" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I44" s="5" t="s">
+      <c r="J44" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J44" s="5" t="s">
+      <c r="K44" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K44" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L44" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M44" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="1">
         <v>244</v>
       </c>
@@ -2555,32 +2690,35 @@
       <c r="D45" s="1">
         <v>80.900000000000006</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="1">
+        <v>47</v>
+      </c>
+      <c r="F45" t="s">
         <v>81</v>
       </c>
-      <c r="F45" s="4" t="s">
+      <c r="G45" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G45" s="4" t="s">
+      <c r="H45" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="H45" s="1" t="s">
+      <c r="I45" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I45" s="5" t="s">
+      <c r="J45" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J45" s="5" t="s">
+      <c r="K45" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K45" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L45" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M45" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="1">
         <v>245</v>
       </c>
@@ -2593,32 +2731,35 @@
       <c r="D46" s="1">
         <v>43.6</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="1">
+        <v>71.2</v>
+      </c>
+      <c r="F46" t="s">
         <v>82</v>
       </c>
-      <c r="F46" s="4" t="s">
+      <c r="G46" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="G46" s="4" t="s">
+      <c r="H46" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="H46" s="1" t="s">
+      <c r="I46" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I46" s="1" t="s">
+      <c r="J46" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="J46" s="1" t="s">
+      <c r="K46" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="K46" s="1" t="s">
+      <c r="L46" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="L46" s="1" t="s">
+      <c r="M46" s="1" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="1">
         <v>246</v>
       </c>
@@ -2631,32 +2772,35 @@
       <c r="D47" s="1">
         <v>90.2</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="1">
+        <v>48.7</v>
+      </c>
+      <c r="F47" t="s">
         <v>83</v>
       </c>
-      <c r="F47" s="4" t="s">
+      <c r="G47" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="G47" s="6" t="s">
+      <c r="H47" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H47" s="5" t="s">
+      <c r="I47" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I47" s="5" t="s">
+      <c r="J47" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J47" s="5" t="s">
+      <c r="K47" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K47" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L47" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M47" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="1">
         <v>247</v>
       </c>
@@ -2669,32 +2813,35 @@
       <c r="D48" s="1">
         <v>90.6</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="1">
+        <v>48.7</v>
+      </c>
+      <c r="F48" t="s">
         <v>84</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="G48" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="G48" s="6" t="s">
+      <c r="H48" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="H48" s="5" t="s">
+      <c r="I48" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="I48" s="5" t="s">
+      <c r="J48" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J48" s="5" t="s">
+      <c r="K48" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K48" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L48" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M48" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="1">
         <v>248</v>
       </c>
@@ -2707,32 +2854,35 @@
       <c r="D49" s="1">
         <v>83</v>
       </c>
-      <c r="E49" t="s">
+      <c r="E49" s="1">
+        <v>45.7</v>
+      </c>
+      <c r="F49" t="s">
         <v>85</v>
       </c>
-      <c r="F49" s="4" t="s">
+      <c r="G49" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="G49" s="4" t="s">
+      <c r="H49" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="H49" s="1" t="s">
+      <c r="I49" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I49" s="5" t="s">
+      <c r="J49" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J49" s="5" t="s">
+      <c r="K49" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="K49" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L49" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M49" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="1">
         <v>249</v>
       </c>
@@ -2745,32 +2895,35 @@
       <c r="D50" s="1">
         <v>86.4</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="1">
+        <v>46.2</v>
+      </c>
+      <c r="F50" t="s">
         <v>86</v>
       </c>
-      <c r="F50" s="4" t="s">
+      <c r="G50" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="G50" s="4" t="s">
+      <c r="H50" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H50" s="1" t="s">
+      <c r="I50" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I50" s="5" t="s">
+      <c r="J50" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J50" s="5" t="s">
+      <c r="K50" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K50" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L50" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M50" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" s="1">
         <v>250</v>
       </c>
@@ -2783,32 +2936,35 @@
       <c r="D51" s="1">
         <v>86</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="1">
+        <v>46.6</v>
+      </c>
+      <c r="F51" t="s">
         <v>87</v>
       </c>
-      <c r="F51" s="4" t="s">
+      <c r="G51" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G51" s="4" t="s">
+      <c r="H51" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="H51" s="1" t="s">
+      <c r="I51" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="I51" s="5" t="s">
+      <c r="J51" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J51" s="5" t="s">
+      <c r="K51" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="K51" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L51" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M51" s="5" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="1">
         <v>251</v>
       </c>
@@ -2821,28 +2977,31 @@
       <c r="D52" s="1">
         <v>73.2</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E52" s="1">
+        <v>45.7</v>
+      </c>
+      <c r="F52" t="s">
         <v>88</v>
       </c>
-      <c r="F52" s="4" t="s">
+      <c r="G52" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="G52" s="4" t="s">
+      <c r="H52" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="H52" s="1" t="s">
+      <c r="I52" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I52" s="5" t="s">
+      <c r="J52" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="J52" s="5" t="s">
+      <c r="K52" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="K52" s="5" t="s">
-        <v>162</v>
-      </c>
       <c r="L52" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="M52" s="5" t="s">
         <v>161</v>
       </c>
     </row>
@@ -2850,7 +3009,7 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A19:D52">
     <sortCondition ref="A19:A52"/>
   </sortState>
-  <conditionalFormatting sqref="C1:D1048576">
+  <conditionalFormatting sqref="C1:E1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>